<commit_message>
feat: add holiday month filtering
</commit_message>
<xml_diff>
--- a/resources/templates/holiday-import-template.xlsx
+++ b/resources/templates/holiday-import-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holidays" sheetId="1" r:id="Ra5c303c3e7034142"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holidays" sheetId="1" r:id="R2516d58634fe455e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -410,7 +410,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="19" t="str">
-        <x:v>Use YYYY-MM-DD dates. Description is optional. Delete the sample row before import.</x:v>
+        <x:v>Use YYYY-MM-DD dates. Description and end_date are optional. A blank end_date uses start_date. Delete the sample row before import.</x:v>
       </x:c>
       <x:c r="B6" s="19"/>
       <x:c r="C6" s="19"/>

</xml_diff>